<commit_message>
Integrate Saidu Ahmed Alkali governance profile
</commit_message>
<xml_diff>
--- a/data/exports/governance_analytics_dataset.xlsx
+++ b/data/exports/governance_analytics_dataset.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -519,27 +519,56 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>54.28</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Evidence-backed weighted score. Use with limitations; missing public data is not proof of poor performance.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>This project is an independent governance analytics and civic-tech research platform based on publicly available information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Dr. Jamilu Isyaku Gwamna</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B4" t="n">
         <v>33.23</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C4" t="n">
         <v>8</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>85.70999999999999</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Evidence-backed weighted score. Use with limitations; missing public data is not proof of poor performance.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>This project is an independent governance analytics and civic-tech research platform based on publicly available information.</t>
         </is>
@@ -556,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1107,6 +1136,251 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>57.73</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>11.55</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>qualitative_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>60.89</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>quantitative_or_mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Youth Empowerment</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>46.24</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>qualitative_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Crisis Handling</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D19" t="n">
+        <v>58.96</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>qualitative_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>qualitative_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Public Utility Management</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>qualitative_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D22" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>qualitative_only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1118,18 +1392,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
@@ -2964,6 +3238,1522 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>EV019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present / Senator for Gombe North</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Official public profile and office history</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>narrative</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>The Federal Ministry of Transportation profile records Alkali's background, Gombe State executive roles, senatorial service, and appointment as Minister of Transportation on 16 August 2023.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Office-history evidence; not a performance outcome by itself.</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>SAID AHMED ALKALI - Honourable Minister of Transportation</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/team/honourable-minister-of-transportation/</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="T20" t="b">
+        <v>1</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>EV020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ministerial performance bond</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>accountability_framework</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>The ministry reported that Alkali signed a performance bond with directors and agency heads to cascade KPIs and annual appraisal for the transportation sector.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Accountability mechanism evidence; implementation outcomes should be monitored over time.</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Transportation Minister Signs Performance Bond With Directors, CEOs, Expresses Readiness To Deliver On Ministerial Mandate</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/transportation-minister-signs-performance-bond-with-directors-ceos-expresses-readiness-to-deliver-on-ministerial-mandate/</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="T21" t="b">
+        <v>1</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EV021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Transport sector economic-enabler policy</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>narrative</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>NITT reported Alkali's position that transport can sustain the economy, reduce unemployment, lower mobility costs, and reduce movement delays for goods and services.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>SRC015</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="M22" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Policy/economic rationale; not a measured GDP statistic.</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Transport Sector Is A Strong Enabler Of The Economy - Hon Minister Of Transportation</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Nigerian Institute of Transport Technology</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>https://nitt.gov.ng/2024/02/11/transport-sector-is-a-strong-enabler-of-the-economy-hon-minister-of-transportation/</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="T22" t="b">
+        <v>1</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>EV022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Kano-Daura rail segment target</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>387</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>kilometres</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Kano Katsina Jigawa Niger corridor</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>The transportation ministry reported Alkali's inspection and assurance on the first 387km Kano-Daura segment of the Kano-Maradi rail project.</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M23" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Project target and inspection evidence; completion must be verified separately.</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>FG Rail Modernization Project: Transport Minister Assures On Completion Of The 387km Kano-Daura Rail Segment By 2025</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/fg-rail-modernization-project-transport-minister-assures-on-completion-of-the-387km-kano-daura-rail-segment-by-2025/</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>68.48</v>
+      </c>
+      <c r="T23" t="b">
+        <v>1</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EV023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Kano-Maradi and Kaduna-Kano rail inspection</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>project_activity</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Northern Nigeria</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>The ministry stated Alkali inspected Kano-Maradi and Kaduna-Kano rail works with engineers, consultants, and contractors for on-ground assessment.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M24" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Inspection and project oversight evidence.</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>FG Rail Modernization Project: Transport Minister Assures On Completion Of The 387km Kano-Daura Rail Segment By 2025</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/fg-rail-modernization-project-transport-minister-assures-on-completion-of-the-387km-kano-daura-rail-segment-by-2025/</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>57.12</v>
+      </c>
+      <c r="T24" t="b">
+        <v>1</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EV024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Lagos-Kano freight restoration plan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>project_activity</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Lagos-Kano corridor</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>The ministry reported plans to restore freight on the Lagos-Kano narrow gauge to support cargo movement to Kano's Dala Inland Dry Port.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M25" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Economic logistics impact is plausible but should be measured through freight-volume data.</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>FG Rail Modernization Project: Transport Minister Assures On Completion Of The 387km Kano-Daura Rail Segment By 2025</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/fg-rail-modernization-project-transport-minister-assures-on-completion-of-the-387km-kano-daura-rail-segment-by-2025/</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>53.04</v>
+      </c>
+      <c r="T25" t="b">
+        <v>1</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>EV025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>National Land Transport Policy approval</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>policy_milestone</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Federal information reporting stated that the first National Land Transport Policy had been validated by stakeholders and approved by the Federal Executive Council.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>SRC017</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M26" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Major policy milestone; full impact depends on implementation.</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Alkali, Transforming Nigeria's Transport Sector</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Information and National Orientation</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>https://fmino.gov.ng/alkali-transforming-nigerias-transport-sector/</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>58.48</v>
+      </c>
+      <c r="T26" t="b">
+        <v>1</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>EV026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Smart mobility and logistics technology agenda</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>policy_activity</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Government information reporting linked Alkali's agenda to smart mobility, intelligent transport systems, blockchain-enabled logistics, NITT logistics-drone testing, and rail unbundling.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>SRC017</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Innovation agenda evidence; measurable deployment metrics should be added as they become available.</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Alkali, Transforming Nigeria's Transport Sector</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Information and National Orientation</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>https://fmino.gov.ng/alkali-transforming-nigerias-transport-sector/</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>53.04</v>
+      </c>
+      <c r="T27" t="b">
+        <v>1</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>EV027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Public Utility Management</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Railway agency performance coordination</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>accountability_framework</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>The performance bond included the Nigerian Railway Corporation and Nigerian Institute of Transport Technology among agencies aligning roles, KPIs, manpower, research, and rail development programmes.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M28" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Public transport institutional management evidence; agency outcomes are multi-actor.</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Transportation Minister Signs Performance Bond With Directors, CEOs, Expresses Readiness To Deliver On Ministerial Mandate</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/transportation-minister-signs-performance-bond-with-directors-ceos-expresses-readiness-to-deliver-on-ministerial-mandate/</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="T28" t="b">
+        <v>1</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>EV028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Crisis Handling</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Railway project delay escalation</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>45</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>percent_completion</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>2023</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Port Harcourt-Aba / Eastern corridor</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Punch reported Alkali criticized the Port Harcourt-Maiduguri contractor after stating work around Port Harcourt-Aba was below expected pace and about 45-47 percent in the inspected section.</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>SRC020</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>regulator_context</t>
+        </is>
+      </c>
+      <c r="M29" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Crisis/implementation response evidence; figure is from reported ministerial inspection comments.</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Port Harcourt-Maiduguri railway: Minister slams contractor, says project disappointing</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Punch Newspapers</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>https://punchng.com/port-harcourt-maiduguri-railway-minister-slams-contractor-says-project-disappointing/</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>58.96</v>
+      </c>
+      <c r="T29" t="b">
+        <v>1</v>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EV029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Public response to railway diversion allegation</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>public_response</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Punch reported the ministry's denial of allegations that a $3bn railway project was diverted to Gombe, and its explanation of project sections and funding constraints.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>SRC019</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="M30" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Represents public controversy and official response; allegation is not treated as proven.</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>$3bn South-East railway project not diverted - Ministry</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Punch Newspapers</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>https://punchng.com/3bn-south-east-railway-project-not-diverted-ministry/</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="T30" t="b">
+        <v>1</v>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>EV030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Transport ministry capital budget release constraint</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>percent_capital_release</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>TheCable reported Alkali saying only about 1 percent of the ministry's 2025 capital budget was released, while 70 percent of projects rolled into 2026 due to funding constraints.</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>SRC018</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>quantitative</t>
+        </is>
+      </c>
+      <c r="M31" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Negative context/constraint, not a personal performance failure.</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Saidu Alkali: Only N2.5bn out of N256.7bn 2025 budget was released to transport ministry</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>TheCable</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>https://www.thecable.ng/saidu-alkali-only-n2-5bn-out-of-n256-7bn-2025-budget-was-released-to-transport-ministry/</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="T31" t="b">
+        <v>1</v>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>source_backed_quantitative</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EV031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Private-sector funding commitments</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>200</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>million_usd</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>TheCable reported a legislative committee statement that the ministry secured private-sector funding commitments of about $200m despite limited capital releases.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>SRC018</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>quantitative</t>
+        </is>
+      </c>
+      <c r="M32" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Attributed to legislative committee comment in reported budget hearing.</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Saidu Alkali: Only N2.5bn out of N256.7bn 2025 budget was released to transport ministry</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>TheCable</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>https://www.thecable.ng/saidu-alkali-only-n2-5bn-out-of-n256-7bn-2025-budget-was-released-to-transport-ministry/</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="T32" t="b">
+        <v>1</v>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>source_backed_quantitative</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>EV032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Kaduna-Kano rail financing and port rail links</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>project_activity</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Kaduna Kano Lagos port corridors</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Independent reported Alkali's statement that financing had been secured for Kaduna-Kano standard gauge and that Badagry, TinCan, Apapa, Lekki, Ijebu Ode and Kajola rail links were initiated.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>SRC021</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M33" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Media report; should be validated against financing agreements and project budgets.</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>FG Secures Financing For Kaduna-Kano Rail Project, Initiates Badagry, TinCan, Apapa Rail Links</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Independent Newspaper Nigeria</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>https://independent.ng/fg-secures-financing-for-kaduna-kano-rail-project-initiates-badagry-tincan-apapa-rail-links/</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="T33" t="b">
+        <v>1</v>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>EV033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Minister of Transportation 2023-present</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Youth Empowerment</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Transport manpower and research mandate through NITT</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>capacity_building</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>2024</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>The ministry reported NITT commitments under the performance bond to provide required manpower, innovation, and transport-sector research.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>project_report</t>
+        </is>
+      </c>
+      <c r="M34" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Institutional capacity-building evidence; no beneficiary count in seed data.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Transportation Minister Signs Performance Bond With Directors, CEOs, Expresses Readiness To Deliver On Ministerial Mandate</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/transportation-minister-signs-performance-bond-with-directors-ceos-expresses-readiness-to-deliver-on-ministerial-mandate/</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="S34" t="n">
+        <v>46.24</v>
+      </c>
+      <c r="T34" t="b">
+        <v>1</v>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>source_backed_contextual</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EV034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Senator / public official</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Public Utility Management</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FERMA oversight context</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>narrative</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>2021</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>A public legislative guide includes Senate committee references involving FERMA and Alkali; direct FERMA agency executive leadership was not verified in the seed public evidence.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>SRC022</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>insufficient_public_evidence</t>
+        </is>
+      </c>
+      <c r="M35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Kept as a research flag because direct FERMA leadership should not be asserted without stronger official source.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Legislative Internship Guide 2021</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Policy and Legal Advocacy Centre</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>https://placng.org/i/wp-content/uploads/2022/04/Legislative-Internship-Guide-2021.pdf</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>secondary_context</t>
+        </is>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>do_not_score_missing_data</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2975,13 +4765,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -3531,6 +5321,426 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>Used only for cross-checking office dates; not used as primary performance evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SAID AHMED ALKALI - Honourable Minister of Transportation</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>government_publication</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/team/honourable-minister-of-transportation/</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Official profile with background, public offices, senatorial service, and ministerial appointment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Transportation Minister Signs Performance Bond With Directors, CEOs, Expresses Readiness To Deliver On Ministerial Mandate</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>government_publication</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2024-02-10</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/transportation-minister-signs-performance-bond-with-directors-ceos-expresses-readiness-to-deliver-on-ministerial-mandate/</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Official ministry report on performance bond, KPI cascade, intermodal transport mandate, and rail programme status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SRC015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Transport Sector Is A Strong Enabler Of The Economy - Hon Minister Of Transportation</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Nigerian Institute of Transport Technology</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>government_publication</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2024-02-11</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://nitt.gov.ng/2024/02/11/transport-sector-is-a-strong-enabler-of-the-economy-hon-minister-of-transportation/</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NITT report on ministerial remarks linking transport to economic growth, jobs, mobility cost, and KPI implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FG Rail Modernization Project: Transport Minister Assures On Completion Of The 387km Kano-Daura Rail Segment By 2025</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>government_publication</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2024-05-10</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/fg-rail-modernization-project-transport-minister-assures-on-completion-of-the-387km-kano-daura-rail-segment-by-2025/</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Official ministry report on inspection of Kano-Maradi and Kaduna-Kano rail projects and freight plans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SRC017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Alkali, Transforming Nigeria's Transport Sector</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Information and National Orientation</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>government_publication</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://fmino.gov.ng/alkali-transforming-nigerias-transport-sector/</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Government information report on National Land Transport Policy, regulatory frameworks, smart mobility, logistics drones, and rail unbundling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SRC018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Saidu Alkali: Only N2.5bn out of N256.7bn 2025 budget was released to transport ministry</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TheCable</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://www.thecable.ng/saidu-alkali-only-n2-5bn-out-of-n256-7bn-2025-budget-was-released-to-transport-ministry/</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Budget-performance report with funding constraints, policy approval, private-sector financing commitments, and legislative challenges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SRC019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>$3bn South-East railway project not diverted - Ministry</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Punch Newspapers</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-03-12</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://punchng.com/3bn-south-east-railway-project-not-diverted-ministry/</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Report on ministry response to public allegation about railway project diversion and funding constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SRC020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Port Harcourt-Maiduguri railway: Minister slams contractor, says project disappointing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Punch Newspapers</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2023-09-22</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://punchng.com/port-harcourt-maiduguri-railway-minister-slams-contractor-says-project-disappointing/</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Report on ministerial inspection, contractor criticism, completion concerns, and public accountability posture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SRC021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>FG Secures Financing For Kaduna-Kano Rail Project, Initiates Badagry, TinCan, Apapa Rail Links</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Independent Newspaper Nigeria</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2024-06-06</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://independent.ng/fg-secures-financing-for-kaduna-kano-rail-project-initiates-badagry-tincan-apapa-rail-links/</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Report on secured financing, Lagos-Kano freight service, port rail links, and transport policy dialogue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SRC022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Legislative Internship Guide 2021</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Policy and Legal Advocacy Centre</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>civil_society_publication</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://placng.org/i/wp-content/uploads/2022/04/Legislative-Internship-Guide-2021.pdf</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>secondary_context</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Public legislative guide used as contextual evidence for Senate committee/FERMA oversight references; direct FERMA agency leadership requires further verification.</t>
         </is>
       </c>
     </row>
@@ -3686,13 +5896,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -3873,31 +6083,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Prof. Isa Ali Ibrahim Pantami</t>
+          <t>Hon. Saidu Ahmed Alkali</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Economy</t>
+          <t>Public Utility Management</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ICT sector GDP contribution</t>
+          <t>FERMA oversight context</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>NCC-linked statement reported ICT contribution to GDP at 14.42 percent in Q2 2021.</t>
+          <t>A public legislative guide includes Senate committee references involving FERMA and Alkali; direct FERMA agency executive leadership was not verified in the seed public evidence.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SRC003</t>
+          <t>SRC022</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.88</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
@@ -3911,17 +6121,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Economy</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Broadband penetration</t>
+          <t>ICT sector GDP contribution</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>NCC-linked statement reported broadband penetration at 40.01 percent by September 2021.</t>
+          <t>NCC-linked statement reported ICT contribution to GDP at 14.42 percent in Q2 2021.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -3949,21 +6159,21 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Broadband access</t>
+          <t>Broadband penetration</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Public report stated 80 million Nigerians had broadband access by December 2021.</t>
+          <t>NCC-linked statement reported broadband penetration at 40.01 percent by September 2021.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SRC011</t>
+          <t>SRC003</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.65</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="9">
@@ -3982,21 +6192,21 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ICT centres established</t>
+          <t>Broadband access</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>USPF ministry-achievements page reported 1667 projects/centres established and 455 ongoing.</t>
+          <t>Public report stated 80 million Nigerians had broadband access by December 2021.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SRC001</t>
+          <t>SRC011</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.78</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="10">
@@ -4010,26 +6220,26 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Innovation</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NITDA institutional development</t>
+          <t>ICT centres established</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>NITDA article credited agency development and GDP relevance in the digital economy ecosystem.</t>
+          <t>USPF ministry-achievements page reported 1667 projects/centres established and 455 ongoing.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SRC002</t>
+          <t>SRC001</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.68</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="11">
@@ -4043,26 +6253,26 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Public Utility Management</t>
+          <t>Innovation</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Utility-sector direct management</t>
+          <t>NITDA institutional development</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>No direct electricity/water utility management role identified in the included public sources.</t>
+          <t>NITDA article credited agency development and GDP relevance in the digital economy ecosystem.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SRC001</t>
+          <t>SRC002</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.2</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="12">
@@ -4076,17 +6286,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Transparency</t>
+          <t>Public Utility Management</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>National identity enrolment</t>
+          <t>Utility-sector direct management</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>USPF ministry-achievements page reported more than 61 million unique NIN enrolments.</t>
+          <t>No direct electricity/water utility management role identified in the included public sources.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -4095,7 +6305,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.76</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
@@ -4109,17 +6319,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Youth Empowerment</t>
+          <t>Transparency</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Digital skills beneficiaries</t>
+          <t>National identity enrolment</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>USPF ministry-achievements page reported more than 219000 direct digital skills beneficiaries.</t>
+          <t>USPF ministry-achievements page reported more than 61 million unique NIN enrolments.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -4128,40 +6338,40 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Economy</t>
+          <t>Youth Empowerment</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Electricity distribution economic contribution</t>
+          <t>Digital skills beneficiaries</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>KEDCO role supports regional commerce through distribution service, but seed data lacks audited economic impact figures.</t>
+          <t>USPF ministry-achievements page reported more than 219000 direct digital skills beneficiaries.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SRC007</t>
+          <t>SRC001</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.35</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="15">
@@ -4175,26 +6385,26 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Economy</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Transformers and feeder construction</t>
+          <t>Electricity distribution economic contribution</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Blueprint reported inspection of new transformers/accessories and feeder construction to improve service delivery.</t>
+          <t>KEDCO role supports regional commerce through distribution service, but seed data lacks audited economic impact figures.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SRC008</t>
+          <t>SRC007</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.68</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="16">
@@ -4208,17 +6418,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Innovation</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Operational modernization</t>
+          <t>Transformers and feeder construction</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Reported transformer/accessory procurement and feeder construction indicate operational improvement activity.</t>
+          <t>Blueprint reported inspection of new transformers/accessories and feeder construction to improve service delivery.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -4227,7 +6437,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="17">
@@ -4241,26 +6451,26 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Public Utility Management</t>
+          <t>Innovation</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kano DisCo metering rate</t>
+          <t>Operational modernization</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NERC Q2 2022 report listed Kano DisCo metering performance at 22.52 percent.</t>
+          <t>Reported transformer/accessory procurement and feeder construction indicate operational improvement activity.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>SRC004</t>
+          <t>SRC008</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.9</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="18">
@@ -4274,26 +6484,26 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Transparency</t>
+          <t>Public Utility Management</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Customer complaints context</t>
+          <t>Kano DisCo metering rate</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>NERC Q4 2022 reported metering, billing, and interruption were major complaint categories across DisCos.</t>
+          <t>NERC Q2 2022 report listed Kano DisCo metering performance at 22.52 percent.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SRC005</t>
+          <t>SRC004</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.82</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="19">
@@ -4307,26 +6517,554 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Customer complaints context</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>NERC Q4 2022 reported metering, billing, and interruption were major complaint categories across DisCos.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SRC005</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Youth Empowerment</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Staff training and retraining</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Daily Trust reported Gwamna statement that staff training and retraining were part of KEDCO transformation strategy.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>SRC007</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G20" t="n">
         <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Crisis Handling</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Railway project delay escalation</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Punch reported Alkali criticized the Port Harcourt-Maiduguri contractor after stating work around Port Harcourt-Aba was below expected pace and about 45-47 percent in the inspected section.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SRC020</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Transport sector economic-enabler policy</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>NITT reported Alkali's position that transport can sustain the economy, reduce unemployment, lower mobility costs, and reduce movement delays for goods and services.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SRC015</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Lagos-Kano freight restoration plan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>The ministry reported plans to restore freight on the Lagos-Kano narrow gauge to support cargo movement to Kano's Dala Inland Dry Port.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Kano-Daura rail segment target</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>The transportation ministry reported Alkali's inspection and assurance on the first 387km Kano-Daura segment of the Kano-Maradi rail project.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Kano-Maradi and Kaduna-Kano rail inspection</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>The ministry stated Alkali inspected Kano-Maradi and Kaduna-Kano rail works with engineers, consultants, and contractors for on-ground assessment.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Kaduna-Kano rail financing and port rail links</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Independent reported Alkali's statement that financing had been secured for Kaduna-Kano standard gauge and that Badagry, TinCan, Apapa, Lekki, Ijebu Ode and Kajola rail links were initiated.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SRC021</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Public Utility Management</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Railway agency performance coordination</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The performance bond included the Nigerian Railway Corporation and Nigerian Institute of Transport Technology among agencies aligning roles, KPIs, manpower, research, and rail development programmes.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Official public profile and office history</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>The Federal Ministry of Transportation profile records Alkali's background, Gombe State executive roles, senatorial service, and appointment as Minister of Transportation on 16 August 2023.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Ministerial performance bond</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>The ministry reported that Alkali signed a performance bond with directors and agency heads to cascade KPIs and annual appraisal for the transportation sector.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Youth Empowerment</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Transport manpower and research mandate through NITT</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>The ministry reported NITT commitments under the performance bond to provide required manpower, innovation, and transport-sector research.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Transport ministry capital budget release constraint</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TheCable reported Alkali saying only about 1 percent of the ministry's 2025 capital budget was released, while 70 percent of projects rolled into 2026 due to funding constraints.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>SRC018</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Private-sector funding commitments</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TheCable reported a legislative committee statement that the ministry secured private-sector funding commitments of about $200m despite limited capital releases.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>SRC018</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>National Land Transport Policy approval</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Federal information reporting stated that the first National Land Transport Policy had been validated by stakeholders and approved by the Federal Executive Council.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SRC017</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Smart mobility and logistics technology agenda</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Government information reporting linked Alkali's agenda to smart mobility, intelligent transport systems, blockchain-enabled logistics, NITT logistics-drone testing, and rail unbundling.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SRC017</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Transparency</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Public response to railway diversion allegation</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Punch reported the ministry's denial of allegations that a $3bn railway project was diverted to Gombe, and its explanation of project sections and funding constraints.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>SRC019</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>0.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand leadership lifecycle analysis
</commit_message>
<xml_diff>
--- a/data/exports/governance_analytics_dataset.xlsx
+++ b/data/exports/governance_analytics_dataset.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>This project is an independent governance analytics and civic-tech research platform based on publicly available information.</t>
+          <t>This platform is an independent civic-tech and governance analytics research project based on publicly available information and evidence-based analysis. It does not represent any political party, candidate, or government institution.</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>This project is an independent governance analytics and civic-tech research platform based on publicly available information.</t>
+          <t>This platform is an independent civic-tech and governance analytics research project based on publicly available information and evidence-based analysis. It does not represent any political party, candidate, or government institution.</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>This project is an independent governance analytics and civic-tech research platform based on publicly available information.</t>
+          <t>This platform is an independent civic-tech and governance analytics research project based on publicly available information and evidence-based analysis. It does not represent any political party, candidate, or government institution.</t>
         </is>
       </c>
     </row>
@@ -4765,16 +4765,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -5741,6 +5741,510 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>Public legislative guide used as contextual evidence for Senate committee/FERMA oversight references; direct FERMA agency leadership requires further verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SRC023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Profile - Prof. Isa Ali Pantami</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Isa Ali Pantami official website</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>biographical_profile</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://isaalipantami.com/biography/</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>self_published_context</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Biographical source for birthplace, education pathway, academic roles, ministerial history and current public profile; used with caution for self-presented claims.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SRC024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Federal government appoints Pantami as DG of NITDA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The Guardian Nigeria</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2016-09-30</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://guardian.ng/technology/federal-government-appoints-pantami-as-dg-of-nitda/</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Contemporary reporting on Pantami's appointment as Director-General of NITDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SRC025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Security experts reject Pantami's plea over pro-Taliban, Al-Qaeda comments</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Punch Newspapers</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2021-04-18</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://punchng.com/security-experts-reject-pantamis-plea-over-pro-taliban-al-qaeda-comments/</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Report on public controversy, criticism and apology/renunciation around past comments attributed to Pantami; used as controversy evidence, not as proof of criminal conduct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SRC026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Professorial Appointment: ASUU Panel Discloses How Pantami Scaled Six Hurdles in FUTO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>THISDAYLIVE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2021-11-08</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2021/11/08/professorial-appointment-asuu-panel-discloses-how-pantami-scaled-six-hurdles-in-futo/</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Reporting on ASUU panel review of Pantami's FUTO professorial appointment controversy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SRC027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Press Release: Alkali's unscheduled inspection of Kubwa Train Station</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>government_publication</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2024-08-27</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://transportation.gov.ng/press-release/</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Official press release on station inspection, accessibility concerns, vandalism response and passenger welfare oversight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SRC028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>I'm Ready to Meet any Customer on Fault Resolution, Says Gwamna</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>THISDAYLIVE</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2016-07-24</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.thisdaylive.com/2016/07/24/im-ready-to-meet-any-customer-on-fault-resolution-says-gwamna-2/</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Report on Gwamna's customer-service and fault-resolution statement as KEDCO MD/CEO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SRC029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Our vision of industrializing, growing economies of KEDCO States is on course - Gwamna</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Economic Confidential</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2019-02-19</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://economicconfidential.com/industrializing-kedco-gwamna/</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Report on Gwamna's stated power-distribution and industrialization vision for KEDCO states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SRC030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Gombe philanthropist sponsors indigenes to study in Moroccan universities</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Vanguard</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2020-01-12</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.vanguardngr.com/2020/01/gombe-philantropist-sponsors-indigenes-to-study-in-moroccan-universities/amp/</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Report on scholarship sponsorship for 10 Gombe students to study in Morocco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SRC031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>How we defeated PDP in Gombe - Gwamna</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Daily Trust</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://dailytrust.com/how-we-defeated-pdp-in-gombe-gwamna/</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>media_interview</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Interview identifying Gwamna as APC chieftain in Gombe State and KEDCO MD/CEO; used only for political-engagement context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SRC032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>What you should know about ministerial nominee: Isa Pantami</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Daily Trust</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://dailytrust.com/what-you-should-know-about-ministerial-nominee-isa-pantami/</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>verified_journalism</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Biographical reporting on Pantami's parents, early Qur'anic education, primary and secondary schooling, university qualifications and early academic career.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SRC033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Sa'idu Ahmed Alkali biography, career, education, life story</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Platinum Times</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>secondary_biographical_profile</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://platinumtimes.ng/saidu-ahmed-alkali-biography-career-education-life-story/</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>secondary_context</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Secondary biographical profile reporting place of birth, community schooling and University of Maiduguri economics education; used cautiously because primary documents were not located.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SRC034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>The magic of KEDCO's revival</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vanguard</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>opinion_media_context</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.vanguardngr.com/2020/02/the-magic-of-kedcos-revival/</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>media_context</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Vanguard-hosted commentary giving Gwamna's academic qualifications and work-experience context; used cautiously as contextual biographical evidence, not audited institutional proof.</t>
         </is>
       </c>
     </row>
@@ -5896,1175 +6400,2607 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>metric_year</t>
+          <t>candidate_name</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>person</t>
+          <t>life_stage</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>year_or_period</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>indicator</t>
+          <t>role_or_event</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>claim_summary</t>
+          <t>institution</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>source_id</t>
+          <t>sector</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>achievement</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>citation</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>impact_category</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>impact_score</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>2019</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Early background</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Publicly unavailable</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Childhood and family background not verified in seed public records</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Personal background</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>No childhood or family-community details are scored because verifiable public records were not located in the seed evidence set.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>The platform does not infer personal background beyond cited public reporting.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SRC006</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Data limitation</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Dr. Jamilu Isyaku Gwamna</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Transparency</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Service delivery pledge</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>TBI Africa reported a service-delivery pledge and staff commitment message by KEDCO MD.</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>SRC009</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2020</v>
-      </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Period not specified</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Accounting and economics qualifications reported</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Ahmadu Bello University; London Metropolitan University</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Vanguard-hosted commentary reported that Gwamna obtained a BSc in Accounting from Ahmadu Bello University, plus an MSc in Business Economics and Finance and a doctorate in Economics from London Metropolitan University.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>This is included as contextual education evidence from media commentary and should be replaced with primary institutional records if available.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SRC034</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Dr. Jamilu Isyaku Gwamna</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Crisis Handling</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>COVID-era electricity service continuity</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Interview stated KEDCO maintained public service delivery during COVID-19 and customers saw improved supply.</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Early career</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>By 2013</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Private-sector utility executive during electricity distribution privatization period</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kano Electricity Distribution Company</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Private-sector leadership</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Daily Trust reporting states that he led KEDCO from its privatization period and described transformation efforts under his leadership.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>This is leadership-context evidence; regulator data is used separately for measurable utility performance.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SRC007</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Private-sector leadership</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Professional growth</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pre-2013</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Multi-sector professional experience reported</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Business and utility-sector institutions</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Private-sector leadership</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Vanguard-hosted commentary reported more than 25 years of work experience across leadership positions before and during KEDCO prominence.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>The dataset treats this as contextual career evidence, not an audited employment chronology.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SRC034</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Professional development</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2016-2022</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Managing Director / Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kano Electricity Distribution Company</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Private-sector leadership</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Multiple journalism sources identify him as MD/CEO of KEDCO.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>The role covers a critical public-utility franchise serving Kano, Katsina and Jigawa states.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>SRC006</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Public utility management</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Dr. Jamilu Isyaku Gwamna</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Public Utility Management</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>KEDCO franchise utility management</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Daily Trust interview described KEDCO service continuity and safety priorities during COVID-19.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>APC political figure in Gombe State</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>All Progressives Congress, Gombe State</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Daily Trust interview identified Gwamna as an APC chieftain in Gombe State and KEDCO MD/CEO.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>This records political engagement; it does not evaluate campaign claims or encourage political persuasion.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>SRC031</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Customer fault-resolution and service-responsiveness pledge</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Kano Electricity Distribution Company</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Public utility management</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>THISDAY reported his stated willingness to meet customers and prioritize fault resolution.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>This is a public service-delivery pledge; measured impact requires complaint-resolution and outage data.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SRC028</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Service delivery</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Power distribution and industrialization vision</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Kano Electricity Distribution Company</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Economic contribution</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Economic Confidential reported his view that reliable power distribution could support industrialization and economic turnaround in KEDCO states.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>This is economic rationale and leadership intent; economic impact is not treated as audited output.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SRC029</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Economic contribution</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>COVID-era service continuity and safety strategy</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kano Electricity Distribution Company</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Crisis handling</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Daily Trust interview reported that KEDCO maintained service delivery during COVID-19 and prioritized safe power supply.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>The claim is interview-based and needs operational supply-hour data for higher confidence.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>SRC006</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Crisis handling</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Community service</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Scholarship support for Gombe students studying in Morocco</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Community philanthropy</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Community service</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Vanguard reported that Gwamna sponsored 10 students from Gombe State to study in Moroccan universities.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>The item is reported philanthropy and scored as community-service evidence, not government performance.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SRC030</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Community service</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Transformer, accessories and feeder construction activity</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Kano Electricity Distribution Company</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Blueprint reported inspections of new transformers, accessories and feeder construction to improve service delivery.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>This is project-activity evidence; completion and reliability gains require independent technical audit.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>SRC008</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Infrastructure development</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Public impact</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Kano DisCo metering rate benchmark</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Nigerian Electricity Regulatory Commission / Kano DisCo</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Public utility management</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NERC Q2 2022 report listed Kano DisCo metering performance at 22.52 percent.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>This is entity-level regulator data and not solely attributable to one executive.</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>SRC004</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Service delivery</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Criticisms and limitations</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Utility-sector performance limitations and complaint context</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kano DisCo / Nigerian electricity distribution sector</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Public perception</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NERC Q4 2022 reported metering, billing and interruption as major complaint categories across DisCos.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>The row captures sector-level public-service constraints and does not assign personal blame without direct evidence.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>SRC005</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Public perception</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Dr. Jamilu Isyaku Gwamna</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Current relevance</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2024-2026</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Public figure associated with utility leadership and Gombe civic philanthropy</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>KEDCO / Gombe civic space</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Current relevance</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Recent app evidence base still identifies him through private-sector utility leadership, political engagement and community-service reporting.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Current relevance is contextual until newer verified public records are added.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>SRC007</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Long-term impact</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Early background</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Born in Gombe State, Nigeria</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Gombe State</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Personal background</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Official transportation ministry profile states that Sai'du Ahmed Alkali was born on February 12, 1969, in Gombe State.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No childhood or family-community narrative is included beyond verified public profile information.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Background context</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Early background</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Family background publicly reported</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Parent identified in secondary public records</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Gombe State</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Family/community background</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Secondary public profiles list Khadi Ahmed Saidu Alkali as his parent.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>This is included cautiously as public biographical context because an official family-source record was not located.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>SRC012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Background context</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Early schooling period</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Community schooling reported</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Gombe community schools</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>A secondary biographical profile reports that Alkali schooled in his community before university.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>This is displayed as secondary-source context and kept at a lower impact score until primary education records are located.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>SRC033</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Period not specified</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Economics degree reported</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>University of Maiduguri</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>A secondary biographical profile reports that Alkali attended the University of Maiduguri and graduated with a degree in Economics.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Education is flagged as secondary-source verified because the official ministry profile does not provide a detailed education timeline.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>SRC033</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Early career</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Before 2010</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Secretary</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Muslim Pilgrims Welfare Board, Gombe State</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Public-sector leadership</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Official profile records early public service as Secretary of the Muslim Pilgrims Welfare Board.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>This marks entry into public-sector administration before elective office.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Institutional leadership</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Professional growth</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Before 2010</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Commissioner of Information</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Gombe State Executive Council</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Public-sector leadership</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Official profile records service as Commissioner of Information in Gombe State.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>The role is included as state-level executive experience; project claims require separate evidence rows.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Public-sector leadership</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2010-2011</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Senator for Gombe North after by-election</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>National Assembly</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Official profile records that he secured the Gombe North senatorial seat after the 2010 by-election.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>This is office-history evidence and not treated as a performance outcome by itself.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2011-2015</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Re-elected Senator for Gombe North</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>National Assembly</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Official profile records continued service after the 2011 general election.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Legislative impact requires bill, committee and constituency-project evidence before stronger scoring.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2019-2023</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Senator for Gombe North under APC</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>National Assembly</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Official profile records re-election in 2019 as a member of the All Progressives Congress.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>This row records public office continuity without campaign messaging or voter persuasion.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Political leadership</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2023-present</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Minister of Transportation</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Ministerial role</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Official profile records appointment as Minister of Transportation on August 16, 2023.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Ministerial impact is assessed through transport policy, rail, logistics and accountability evidence rows.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>SRC013</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Ministerial leadership</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Kano-Maradi and Kaduna-Kano rail project inspections</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>The ministry reported inspections of Kano-Maradi and Kaduna-Kano rail works and assurance on the 387km Kano-Daura segment.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>The row captures project oversight and stated targets; completion and value-for-money require further project records.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>SRC016</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Infrastructure development</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Performance bond and KPI cascade</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation and agencies</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Governance reform</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>The ministry reported a performance bond with directors and agency heads to cascade KPIs and annual appraisal.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>This is an accountability mechanism; implementation outcomes should be monitored over time.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>SRC014</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Governance efficiency</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>National Land Transport Policy approval</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation / Federal Executive Council</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Policy reform</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Government information reporting stated the first National Land Transport Policy had been validated and approved by the Federal Executive Council.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>This is a major policy milestone; measurable impact depends on implementation and sector outcome tracking.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>SRC017</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Policy reform</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Criticisms and controversies</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2023-2025</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Rail implementation delays and public allegations</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Railway project corridors</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Public controversy</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Journalism reported contractor criticism over delayed railway work and a ministry denial of allegations that a railway project was diverted.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>The allegation is not treated as proven; the dataset records both public criticism and official response.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>SRC019</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Public perception</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Public impact</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Budget-release constraint and private financing context</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Economic governance</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>TheCable reported the minister saying only about one percent of the 2025 capital budget had been released, while a legislative committee cited about $200m in private-sector commitments.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>This is treated as policy-context evidence and funding constraint, not a personal performance failure.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>SRC018</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Economic contribution</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Hon. Saidu Ahmed Alkali</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Current relevance</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2024-2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Transport reform, accessibility and rail-service oversight</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Transportation / NRC</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Current relevance</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Ministry press material records station inspections covering vandalism, accessibility and passenger welfare concerns.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Current relevance is tied to ongoing transport service delivery and institutional supervision.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>SRC027</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Public impact</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Prof. Isa Ali Ibrahim Pantami</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Crisis Handling</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>COVID-era digital economy continuity</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ICT sector growth during the recession period was cited in official achievements materials.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Early background</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Born in Pantami, Gombe State, Nigeria</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Pantami community, Gombe State</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Personal background</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Publicly available profiles identify his birthplace as Pantami in Gombe State.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Official and biographical profiles record Pantami as born in Pantami, Gombe State; no independently verified childhood narrative is included in this dataset.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>SRC023</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Background context</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Early background</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Family background publicly reported</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pantami community, Gombe State</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Family/community background</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Daily Trust reported that Pantami was born to Malama Amina Umar Aliyu and Malam Ali Ibrahim Pantami.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>This personal-background row is included because it is publicly reported by a reputable newspaper; no private family details beyond the public report are added.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>SRC032</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Background context</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Childhood-1980s</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Qur'anic and primary education</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Tsangaya School; Pantami Primary School</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Daily Trust reported that Pantami started with Tsangaya Qur'anic education and later attended Pantami Primary School.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>This gives users early-life context without inventing unsupported childhood narrative.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>SRC032</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2003-2008</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Computer science university qualifications</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Abubakar Tafawa Balewa University</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Daily Trust and his public biography report a BTech in Computer Science in 2003 and a master's degree in 2008 from ATBU.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Education history is treated as verified biographical context, not a governance outcome by itself.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>SRC032</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Post-2008</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Doctoral qualification</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Robert Gordon University, Aberdeen</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Public profiles report that Pantami obtained a PhD from Robert Gordon University in Scotland.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>The dataset records the qualification and avoids broader claims about merit beyond the source.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>SRC023</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Secondary school period</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Secondary education</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Government Science Secondary School, Gombe</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Daily Trust reported that Pantami obtained his SSCE from Government Science Secondary School, Gombe.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>This is treated as education-history context, not a governance performance outcome.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>SRC032</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Early career</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2000s-2014</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Lecturer and academic in information technology</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Abubakar Tafawa Balewa University</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Academic leadership</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Taught undergraduate and postgraduate information technology courses for more than a decade according to his public biography.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>This supports academic and professional formation before national public office.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>SRC023</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Professional development</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Professional growth</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2014-2016</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Academic role in computing and information systems</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Islamic University of Madinah</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Academic leadership</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Public biography records an international academic role before his appointment to NITDA.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>The role is included as professional experience; this dataset does not infer institutional impact without independent metrics.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>SRC023</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Professional development</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2016-2019</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Director-General / CEO</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>National Information Technology Development Agency</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Public-sector leadership</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Appointed to lead NITDA in 2016.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>The appointment is documented in contemporary public reporting; performance impacts are scored only where evidence rows exist in the evidence ledger.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>SRC024</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Institutional leadership</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Major leadership roles</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2019-2023</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Minister of Communications and Digital Economy</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Communications and Digital Economy</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Ministerial role</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Served as minister after the communications portfolio was expanded to digital economy.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Official achievement documents and policy papers connect this period with digital economy policy, broadband and identity-management programmes.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>SRC001</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Public Utility Management</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>FERMA oversight context</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>A public legislative guide includes Senate committee references involving FERMA and Alkali; direct FERMA agency executive leadership was not verified in the seed public evidence.</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>SRC022</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Public-sector leadership</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Prof. Isa Ali Ibrahim Pantami</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ICT sector GDP contribution</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>NCC-linked statement reported ICT contribution to GDP at 14.42 percent in Q2 2021.</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2019-2021</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Digital skills and ICT access programmes</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Communications and Digital Economy / USPF</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Policy and projects</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>USPF-linked achievement material reported more than 219000 direct digital-skills beneficiaries and 1667 ICT centres/projects established.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>These are government-reported outputs and should be read as programme indicators, not audited personal-only achievements.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>SRC001</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Service delivery</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Major achievements</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2020-2030 policy period</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>National Digital Economy Policy and Strategy</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Communications and Digital Economy</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Policy reform</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>The National Digital Economy Policy and Strategy set an eight-pillar framework for Nigeria's digital economy agenda.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Policy existence is verifiable; implementation impact is evaluated through separate evidence rows and measurable indicators.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>SRC010</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Policy reform</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Prof. Isa Ali Ibrahim Pantami</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Public impact</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ICT sector GDP and broadband indicators</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>NCC / communications sector</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Economic and infrastructure outcomes</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>NCC-linked reporting stated ICT contributed 14.42 percent to GDP in Q2 2021 and broadband penetration reached 40.01 percent by September 2021.</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>The dataset attributes these as sector outcomes under a multi-actor regulatory and market ecosystem, not sole-person causation.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
         <is>
           <t>SRC003</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>0.88</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Economic contribution</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Prof. Isa Ali Ibrahim Pantami</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Broadband penetration</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>NCC-linked statement reported broadband penetration at 40.01 percent by September 2021.</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>SRC003</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>0.88</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Criticisms and controversies</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Professorship appointment controversy and review</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Federal University of Technology Owerri / ASUU discourse</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Academic controversy</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Media reporting described public debate over his FUTO professorial appointment and later reporting on an ASUU panel review.</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>The row is included for balanced lifecycle analysis; it is not scored as a governance achievement.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>SRC026</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Public perception</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Prof. Isa Ali Ibrahim Pantami</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Broadband access</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Public report stated 80 million Nigerians had broadband access by December 2021.</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>SRC011</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>0.65</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Criticisms and controversies</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Public controversy over past extremist comments</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Public media and civic debate</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Public controversy</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Reputable journalism reported controversy over past comments attributed to Pantami and reported that he renounced or apologized for earlier views.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>This row records the controversy as reported public perception; it does not present allegations as proven criminal conduct.</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>SRC025</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Public perception</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Prof. Isa Ali Ibrahim Pantami</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>ICT centres established</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>USPF ministry-achievements page reported 1667 projects/centres established and 455 ongoing.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>SRC001</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Prof. Isa Ali Ibrahim Pantami</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Innovation</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>NITDA institutional development</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>NITDA article credited agency development and GDP relevance in the digital economy ecosystem.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>SRC002</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Prof. Isa Ali Ibrahim Pantami</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Public Utility Management</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Utility-sector direct management</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>No direct electricity/water utility management role identified in the included public sources.</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>SRC001</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Prof. Isa Ali Ibrahim Pantami</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Transparency</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>National identity enrolment</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>USPF ministry-achievements page reported more than 61 million unique NIN enrolments.</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>SRC001</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>0.76</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Prof. Isa Ali Ibrahim Pantami</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Youth Empowerment</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Digital skills beneficiaries</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>USPF ministry-achievements page reported more than 219000 direct digital skills beneficiaries.</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>SRC001</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Electricity distribution economic contribution</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>KEDCO role supports regional commerce through distribution service, but seed data lacks audited economic impact figures.</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>SRC007</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Transformers and feeder construction</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Blueprint reported inspection of new transformers/accessories and feeder construction to improve service delivery.</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>SRC008</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Innovation</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Operational modernization</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Reported transformer/accessory procurement and feeder construction indicate operational improvement activity.</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>SRC008</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>0.58</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Public Utility Management</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Kano DisCo metering rate</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>NERC Q2 2022 report listed Kano DisCo metering performance at 22.52 percent.</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>SRC004</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Transparency</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Customer complaints context</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>NERC Q4 2022 reported metering, billing, and interruption were major complaint categories across DisCos.</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>SRC005</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>0.82</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Dr. Jamilu Isyaku Gwamna</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Youth Empowerment</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Staff training and retraining</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Daily Trust reported Gwamna statement that staff training and retraining were part of KEDCO transformation strategy.</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>SRC007</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Crisis Handling</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Railway project delay escalation</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Punch reported Alkali criticized the Port Harcourt-Maiduguri contractor after stating work around Port Harcourt-Aba was below expected pace and about 45-47 percent in the inspected section.</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>SRC020</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Transport sector economic-enabler policy</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>NITT reported Alkali's position that transport can sustain the economy, reduce unemployment, lower mobility costs, and reduce movement delays for goods and services.</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>SRC015</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Lagos-Kano freight restoration plan</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>The ministry reported plans to restore freight on the Lagos-Kano narrow gauge to support cargo movement to Kano's Dala Inland Dry Port.</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>SRC016</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Kano-Daura rail segment target</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>The transportation ministry reported Alkali's inspection and assurance on the first 387km Kano-Daura segment of the Kano-Maradi rail project.</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>SRC016</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>0.86</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Kano-Maradi and Kaduna-Kano rail inspection</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>The ministry stated Alkali inspected Kano-Maradi and Kaduna-Kano rail works with engineers, consultants, and contractors for on-ground assessment.</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>SRC016</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>0.84</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Infrastructure</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Kaduna-Kano rail financing and port rail links</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Independent reported Alkali's statement that financing had been secured for Kaduna-Kano standard gauge and that Badagry, TinCan, Apapa, Lekki, Ijebu Ode and Kajola rail links were initiated.</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>SRC021</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Public Utility Management</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Railway agency performance coordination</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>The performance bond included the Nigerian Railway Corporation and Nigerian Institute of Transport Technology among agencies aligning roles, KPIs, manpower, research, and rail development programmes.</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>SRC014</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>0.76</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Transparency</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Official public profile and office history</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>The Federal Ministry of Transportation profile records Alkali's background, Gombe State executive roles, senatorial service, and appointment as Minister of Transportation on 16 August 2023.</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>SRC013</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Transparency</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Ministerial performance bond</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>The ministry reported that Alkali signed a performance bond with directors and agency heads to cascade KPIs and annual appraisal for the transportation sector.</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>SRC014</t>
-        </is>
-      </c>
-      <c r="G29" t="n">
-        <v>0.82</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Youth Empowerment</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Transport manpower and research mandate through NITT</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>The ministry reported NITT commitments under the performance bond to provide required manpower, innovation, and transport-sector research.</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>SRC014</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>0.68</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Transport ministry capital budget release constraint</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>TheCable reported Alkali saying only about 1 percent of the ministry's 2025 capital budget was released, while 70 percent of projects rolled into 2026 due to funding constraints.</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>SRC018</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>0.82</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Private-sector funding commitments</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>TheCable reported a legislative committee statement that the ministry secured private-sector funding commitments of about $200m despite limited capital releases.</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>SRC018</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Innovation</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>National Land Transport Policy approval</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Federal information reporting stated that the first National Land Transport Policy had been validated by stakeholders and approved by the Federal Executive Council.</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>SRC017</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>0.86</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Innovation</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Smart mobility and logistics technology agenda</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Government information reporting linked Alkali's agenda to smart mobility, intelligent transport systems, blockchain-enabled logistics, NITT logistics-drone testing, and rail unbundling.</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>SRC017</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Hon. Saidu Ahmed Alkali</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Transparency</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Public response to railway diversion allegation</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Punch reported the ministry's denial of allegations that a $3bn railway project was diverted to Gombe, and its explanation of project sections and funding constraints.</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>SRC019</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>0.66</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Current relevance</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2024-2026</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Author, public speaker and digital policy figure</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Public policy and technology discourse</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Current relevance</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Public profiles and reporting continue to identify Pantami with digital economy, cybersecurity and public-policy debates.</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Current relevance is treated as contextual because post-ministerial outcomes require fresh source verification before scoring.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>SRC023</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Long-term impact</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>